<commit_message>
docs(venue): renumber withdrawal decisions after review
Refs SCRUM-47 / E06-S03; address #280 review without closing the story. Reserve T-93 for #279; use T-94 through T-96 and regenerate CAA 161026 exports. Preserve current sprint labels pending planning confirmation.
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES.xlsx
+++ b/docs/testing/PROJECT TEST CASES.xlsx
@@ -9327,7 +9327,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>E06-S03 — Scenario 3 (Several venue bookings for one event); Scenario 3b (Bookings may cover different windows inside the event); confirmed O-29 (T-78); Pending-only withdrawal and requested-venue notices (T-93, T-94)</t>
+          <t>E06-S03 — Scenario 3 (Several venue bookings for one event); Scenario 3b (Bookings may cover different windows inside the event); confirmed O-29 (T-78); Pending-only withdrawal and requested-venue notices (T-94, T-95)</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -9379,7 +9379,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>E06-S03 — Scenario 3e; T-93, T-94</t>
+          <t>E06-S03 — Scenario 3e; T-94, T-95</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -9431,7 +9431,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>E06-S03 — Scenario 3e; T-94</t>
+          <t>E06-S03 — Scenario 3e; T-95</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>E06-S03 — Scenario 3e; T-93, T-94</t>
+          <t>E06-S03 — Scenario 3e; T-94, T-95</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -9536,7 +9536,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>E06-S03 — Scenario 3e, 3f; T-94, T-95</t>
+          <t>E06-S03 — Scenario 3e, 3f; T-95, T-96</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>E06-S03 — Scenario 3f; T-95</t>
+          <t>E06-S03 — Scenario 3f; T-96</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(testing): regenerate three-precondition testcase exports
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES.xlsx
+++ b/docs/testing/PROJECT TEST CASES.xlsx
@@ -8486,7 +8486,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>Venue "Riverside Hall" has Turnaround time 0; Confirmed bookings exist for "Charity Run" 15/01/2027 10:00-12:00 (coordinator_1) and "Alumni Dinner" 15/01/2027 12:30-14:00 (coordinator_2); venue_staff_1@connectsphere.com is signed in</t>
+          <t>Venue "Riverside Hall" has Setup time 0 and Turnaround time 0 before either booking is created; Confirmed bookings exist for "Charity Run" 15/01/2027 10:00-12:00 (coordinator_1) and "Alumni Dinner" 15/01/2027 12:30-14:00 (coordinator_2); venue_staff_1@connectsphere.com is signed in</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -10381,7 +10381,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>Venue "Riverside Hall" has Setup time 30 and Turnaround time 45; "Charity Run" is Confirmed 15/01/2027 10:00-12:00; a Pending request for "Alumni Dinner" 15/01/2027 12:30-14:00 was created before the buffers were set; venue_staff_1@connectsphere.com is signed in</t>
+          <t>Venue "Riverside Hall" initially has Setup time 0 and Turnaround time 0 when both bookings are created: "Charity Run" is Confirmed 15/01/2027 10:00-12:00 and "Alumni Dinner" is Pending 15/01/2027 12:30-14:00. Then Setup time is set to 30 and Turnaround time to 45, retaining both bookings; venue_staff_1@connectsphere.com is signed in</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>Venue Orchid Hall has a confirmed booking for 2026-11-10 09:00:00 to 2026-11-10 11:00:00. A pending request exists for the same venue for 2026-11-10 11:00:00 to 2026-11-10 13:00:00</t>
+          <t>Venue Orchid Hall has Setup time 0 and Turnaround time 0 before either booking is created. It has a confirmed booking for 2026-11-10 09:00:00 to 2026-11-10 11:00:00. A pending request exists for the same venue for 2026-11-10 11:00:00 to 2026-11-10 13:00:00</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(testing): reconcile E06-S06 rule-B cases
E06-S06 / SCRUM-50. Preserve all seven case IDs, replace impossible overlaps with real buffer-change fixtures and regenerate the dated/current catalogue.
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES.xlsx
+++ b/docs/testing/PROJECT TEST CASES.xlsx
@@ -10939,7 +10939,7 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 1 (Overlapping approval blocked)</t>
+          <t>E06-S06 - Scenario 4 (Approval rechecks current buffered availability; T-100)</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -10954,29 +10954,28 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>Verify that attempting to approve a request that overlaps an existing confirmed booking for the same venue should be blocked with the conflicting booking identified</t>
+          <t>Verify approval rechecks a confirmed booking after buffer growth</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>"Riverside Hall" has a confirmed booking for "Charity Run" on 15/01/2027, 09:00-17:00. A second pending request for "Riverside Hall" on 15/01/2027, 14:00-18:00 exists for event "Product Expo 2026"</t>
+          <t>Venue Orchid Hall has setup and turnaround set to 0. Confirmed booking Charity Run occupies 09:00-11:00 and Pending request Product Expo occupies 11:00-13:00; both were accepted while their advertised periods were adjacent. Venue Staff then changes setup time to 30 minutes.</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
-          <t>1. Log in as venue_staff_1@connectsphere.com
-  2. Open the pending request for "Product Expo 2026"
-  3. Attempt to click "Approve"</t>
+          <t>1. Confirm the buffer edit saves and affected bookings remain present with the `buffer_conflict` flag.
+2. Open Product Expo's Pending request and attempt approval.</t>
         </is>
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>Existing confirmed booking: Charity Run, 15/01/2027 09:00-17:00 | Conflicting request: Product Expo 2026, 15/01/2027 14:00-18:00</t>
+          <t>Before edit: Charity Run 09:00-11:00; Product Expo 11:00-13:00; both buffers 0. After edit: setup 30 minutes creates a 10:30-11:00 overlap between their buffered windows.</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>Approval is blocked, and the message identifies the existing confirmed "Charity Run" booking as the conflict</t>
+          <t>Approval is refused after checking current buffers. The Confirmed booking and Pending request are retained, their conflict remains flagged, and neither is silently released.</t>
         </is>
       </c>
     </row>
@@ -10991,7 +10990,7 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 2 (Competing request flagged)</t>
+          <t>E06-S06 - Scenario 2 (Later overlapping claim refused; T-100)</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -11006,29 +11005,28 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>Verify that approving one of two pending requests for the same venue and overlapping times should flag the other as conflicting</t>
+          <t>Verify a later overlapping request is refused while the first claim remains active</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>Two pending requests exist for "Riverside Hall" on 20/01/2027, both 09:00-12:00: Request A ("Tech Conference 2026") and Request B ("Product Expo 2026")</t>
+          <t>Orchid Hall has no active booking. The setup and turnaround buffers are 30 and 45 minutes. A successfully accepted Pending request for Charity Run occupies advertised time 09:00-11:00.</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>1. Log in as venue_staff_1@connectsphere.com
-  2. Approve Request A ("Tech Conference 2026")
-  3. Open Request B ("Product Expo 2026")</t>
+          <t>1. Submit a normal booking request for Product Expo at 10:00-12:00 on Orchid Hall.
+2. Read the original request and the venue's booking list.</t>
         </is>
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>Request A: Tech Conference 2026 (approved) | Request B: Product Expo 2026 (same venue, overlapping time)</t>
+          <t>First accepted claim: Charity Run, 09:00-11:00. Later overlapping request: Product Expo, 10:00-12:00, same venue.</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>Request B is now flagged as conflicting and cannot be approved until the conflict is resolved</t>
+          <t>The second request is refused while Charity Run's claim is active. Charity Run remains unchanged and no overlapping Pending row is created.</t>
         </is>
       </c>
     </row>
@@ -11043,12 +11041,12 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 3 (Simultaneous approval fails safely)</t>
+          <t>E06-S06 - Scenario 3 (Concurrent claims fail safely; T-100)</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>4 - Negative</t>
+          <t>3 - Integration / regression</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr">
@@ -11058,28 +11056,28 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>Verify that if another Venue Staff member approves a conflicting request moments earlier, a simultaneous approval attempt should fail safely and inform the user the venue has just been taken</t>
+          <t>Verify concurrent overlapping new claims accept only one request</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>Two pending requests exist for "Riverside Hall" on 25/01/2027, overlapping times. venue_staff_2@connectsphere.com approves one of them a moment before venue_staff_1@connectsphere.com processes the other</t>
+          <t>Orchid Hall has no active booking and has 30-minute setup and 45-minute turnaround buffers. Two assigned Coordinators for separate Approved events submit overlapping booking requests concurrently.</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
-          <t>1. As venue_staff_2@connectsphere.com, approve Request A for "Riverside Hall" on 25/01/2027
-  2. Immediately as venue_staff_1@connectsphere.com, attempt to approve the conflicting Request B for the same venue and overlapping time</t>
+          <t>1. Submit both requests in parallel transactions for the same venue.
+2. Read both responses, booking rows, event statuses, notifications and audit effects.</t>
         </is>
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>Request A approved by venue_staff_2@connectsphere.com just before venue_staff_1@connectsphere.com's attempt on Request B</t>
+          <t>Request A: Charity Run, 09:00-11:00. Request B: Product Expo, 10:00-12:00. Both target Orchid Hall.</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>venue_staff_1@connectsphere.com's approval attempt fails safely, with a message stating the venue has just been taken by another approval</t>
+          <t>Exactly one request is accepted. The loser receives 409; it creates no booking row, event-status change, notification or audit effect. Only the accepted request's effects remain.</t>
         </is>
       </c>
     </row>
@@ -11094,7 +11092,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 · Scenario 1 (Overlapping approval blocked)</t>
+          <t>E06-S06 - Scenario 4 (Approval rechecks current buffered availability; T-100)</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -11109,29 +11107,28 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>Verify that a booking beginning exactly when another ends is not treated as a conflict</t>
+          <t>Verify exact half-open buffered adjacency is allowed with zero buffers</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>Venue Orchid Hall has a confirmed booking for 2026-11-10 09:00:00 to 2026-11-10 11:00:00. A pending request exists for the same venue for 2026-11-10 11:00:00 to 2026-11-10 13:00:00</t>
+          <t>Orchid Hall has setup and turnaround set to 0. It has a Confirmed booking for Charity Run from 09:00 to 11:00 and an accepted Pending request for Product Expo from 11:00 to 13:00.</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
-          <t>1. Sign in as Venue Staff
- 2. Open the pending request for 11:00–13:00
- 3. Approve it</t>
+          <t>1. Open the Pending Product Expo request.
+2. Approve it and read both bookings on the venue calendar.</t>
         </is>
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>Existing: 09:00–11:00 · Requested: 11:00–13:00 · Shared boundary: 11:00</t>
+          <t>Existing: 09:00-11:00. Requested: 11:00-13:00. Both buffers: 0. Shared half-open boundary: 11:00.</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>The approval succeeds and both bookings show as Confirmed on the venue calendar. Ranges are half-open, so touching at the boundary is not an overlap</t>
+          <t>Approval succeeds and both bookings are Confirmed. The exact half-open boundary is adjacent, not overlapping.</t>
         </is>
       </c>
     </row>
@@ -11146,7 +11143,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 · Scenario 1 (Overlapping approval blocked)</t>
+          <t>E06-S06 - Scenario 4 (Approval rechecks current buffered availability; T-100)</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -11161,29 +11158,28 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>Verify that a booking overlapping an existing one by a single minute is blocked</t>
+          <t>Verify a one-minute overlap is refused before an impossible fixture is inserted</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>Venue Orchid Hall has a confirmed booking for 2026-11-10 09:00:00 to 2026-11-10 11:00:00. A pending request exists for the same venue for 2026-11-10 10:59:00 to 2026-11-10 13:00:00</t>
+          <t>Orchid Hall has setup and turnaround set to 0 and one active Confirmed booking for Charity Run from 09:00 to 11:00. No Pending request exists for a conflicting period.</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
-          <t>1. Sign in as Venue Staff
- 2. Open the pending request for 10:59–13:00
- 3. Attempt to approve it</t>
+          <t>1. Submit a new booking request for Product Expo from 10:59 to 13:00 on Orchid Hall.
+2. Read the response and the venue's booking rows.</t>
         </is>
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>Existing: 09:00–11:00 · Requested: 10:59–13:00 · Overlap: 1 minute</t>
+          <t>Existing claim: 09:00-11:00. Attempted request: 10:59-13:00. Advertised overlap: 1 minute. Both buffers: 0.</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>Approval is blocked and the conflicting 09:00–11:00 booking is identified. The venue never holds two confirmed bookings over the same period</t>
+          <t>The new request is refused at submission and no overlapping Pending fixture is inserted. The Coordinator is told that the requested buffered window is unavailable, without disclosure of another event's title or private booking details. Charity Run's prior claim remains unchanged.</t>
         </is>
       </c>
     </row>
@@ -11198,7 +11194,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 — Scenario 4 (Buffered windows are what must not overlap)</t>
+          <t>E06-S06 - Scenario 4 (Approval rechecks current buffered availability; T-100)</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -11213,28 +11209,30 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>Verify that two approvals whose advertised times do not overlap but whose buffered windows do should let at most one succeed when processed at the same moment</t>
+          <t>Verify buffer-growth conflicts block approvals until an explicit resolution</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>Venue "Riverside Hall" has Setup time 30 and Turnaround time 45; two Pending requests exist on it for 15/01/2027: "Charity Run" 10:00-12:00 and "Alumni Dinner" 12:30-14:00; two Venue Staff accounts are signed in; TEST_DATABASE_URL points at the disposable test schema</t>
+          <t>Orchid Hall has setup and turnaround set to 0. Two Pending requests, Charity Run 10:00-12:00 and Alumni Dinner 12:00-14:00, were successfully accepted while their advertised windows were adjacent. Venue Staff then changes setup to 30 minutes and turnaround to 45 minutes.</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>1. Trigger approval of both requests concurrently (integration test issues both approvals in parallel transactions)
-  2. Read back both bookings and the venue calendar</t>
+          <t>1. Confirm the buffer edit saves, both Pending rows remain, and both show `buffer_conflict`.
+2. Attempt approval of each request while the buffered conflict remains.
+3. Resolve the conflict using one of these paths: (primary) Venue Staff reject one conflicting Pending request with a reason; (alternative) an authorized Coordinator withdraws/replans one request to a nonconflicting period and resubmits it as needed.
+4. Approve the remaining now-free Pending request. For the alternative path, also approve the replanned request only if it is Pending and conflict-free.</t>
         </is>
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>Charity Run buffered: 09:30-12:45 | Alumni Dinner buffered: 12:00-14:45 (advertised times do not overlap; buffered windows overlap 12:00-12:45)</t>
+          <t>Initially both buffers are 0. After the edit, Charity Run occupies 09:30-12:45 and Alumni Dinner occupies 11:30-14:45; these windows overlap from 11:30 to 12:45.</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>Exactly one booking is Confirmed; the other approval fails with the conflict identified and its request remains Pending; the database exclusion constraint rejected the second write on the buffered range (ADR-003), so TC_E06S06_04 (adjacent, must not conflict) and TC_E06S06_05 (one minute of overlap) continue to hold on buffered windows</t>
+          <t>Both approvals are refused while the conflict remains, and there is no automatic winner. The primary resolution is for Venue Staff to reject one conflicting Pending request with a reason; that row becomes terminal Rejected, and the remaining still-Pending request can then be approved. Alternatively, an authorized Coordinator may withdraw/replan one request to a nonconflicting period; the remaining now-free Pending request and any valid replanned Pending request can then be approved. A Rejected row is never approved.</t>
         </is>
       </c>
     </row>
@@ -11249,7 +11247,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 — Scenario 5 (Conflicts are per venue, not per event)</t>
+          <t>E06-S06 - Scenario 5 (Conflicts are per venue, not per event; T-100)</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -11264,29 +11262,29 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>Verify that approving two requests from the same event on two different venues over the same period should confirm both</t>
+          <t>Verify one event may confirm overlapping bookings at different venues</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>Event "Tech Summit" has Pending requests on "Seminar Room A" and "Seminar Room B" for 15/01/2027 14:00-16:00 (TC_E06S03_07); venue_staff_1@connectsphere.com is signed in</t>
+          <t>Event Tech Summit has accepted Pending requests on Seminar Room A and Seminar Room B for 15/01/2027 14:00-16:00 (TC_E06S03_07). Each venue has no conflicting active booking.</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>1. Approve the "Seminar Room A" request
-  2. Approve the "Seminar Room B" request
-  3. Open the availability calendar for both venues on 15/01/2027</t>
+          <t>1. Approve the Seminar Room A request.
+2. Approve the Seminar Room B request.
+3. Read both venue calendars.</t>
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>Same event, same period, two venues</t>
+          <t>Same event and period; different venues.</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>Both bookings become Confirmed; neither approval is blocked; each venue's calendar shows its own Confirmed period; TC_E06S06_01 to TC_E06S06_06 (conflicts on one venue) continue to hold</t>
+          <t>Both requests are accepted and become Confirmed. Each venue calendar shows its own booking; neither venue's availability check blocks the other. E06-S03's multiple-venue semantics remain unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(testing): align the E08-S04 test cases with the acceptance criteria (SCRUM-235)
- TC_E08S04_05: drop the leftover second version (manual "Submit for safety
  check"), which contradicted Scenario 4 and filled the exported row; the case
  now also reads the Activity log for the kept earlier approval.
- TC_E08S04_03: check "Revert to Planning" is still offered (Scenario 3), in
  the case, the guide and the Playwright test.
- TC_E08S04_04: read the Coordinator's Activity log; the app has no System
  Administrator role.
- Click-through: steps B-5 and C-9. Test cases re-exported (CAA 311026).
- Handoff: E08-S06 interactions for its builder.
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES.xlsx
+++ b/docs/testing/PROJECT TEST CASES.xlsx
@@ -14023,7 +14023,8 @@
       <c r="H259" s="2" t="inlineStr">
         <is>
           <t>1. Open Leadership Summit
-2. Review its status and technical arrangement warning</t>
+2. Review its status and technical arrangement warning
+3. Check the actions offered to the Coordinator</t>
         </is>
       </c>
       <c r="I259" s="2" t="inlineStr">
@@ -14033,7 +14034,7 @@
       </c>
       <c r="J259" s="2" t="inlineStr">
         <is>
-          <t>The Event stays Confirmed; the technical arrangement is flagged for review; no automatic status change occurs under this rule</t>
+          <t>The Event stays Confirmed; the technical arrangement is flagged for review; no automatic status change occurs under this rule; "Revert to Planning" is still offered to the Coordinator</t>
         </is>
       </c>
     </row>
@@ -14073,8 +14074,8 @@
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
-          <t>1. Log in as a System Administrator
-  2. Open the Activity Log and search for "Leadership Summit"</t>
+          <t>1. Log in as coordinator_1@connectsphere.com
+  2. Open event "Leadership Summit" and read its Activity log</t>
         </is>
       </c>
       <c r="I260" s="2" t="inlineStr">
@@ -14084,7 +14085,7 @@
       </c>
       <c r="J260" s="2" t="inlineStr">
         <is>
-          <t>An activity log entry exists recording the reversion, with actor = coordinator_1@connectsphere.com, action = "Reverted to Planning", and a timestamp</t>
+          <t>An activity log entry exists recording the reversion, with actor = coordinator_1 (shown by name), action = "Reverted to Planning", and a timestamp</t>
         </is>
       </c>
     </row>
@@ -14119,24 +14120,24 @@
       </c>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t>Event "Charity Run" was Confirmed through a safety approval, then reverted to Planning by coordinator_1 with a reason; its arrangements are complete again</t>
+          <t>Event Charity Run was Confirmed through a safety approval, then returned to Planning; all required venue and technical arrangements are being reconfirmed</t>
         </is>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
-          <t>1. As coordinator_1, click "Submit for safety check"
-  2. Read the status and the activity log
-  3. As safety_1@connectsphere.com, approve the event</t>
+          <t>1. Confirm the final required venue or technical arrangement
+2. Read the Event status and notifications
+3. Read the Event's Activity log</t>
         </is>
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>Second pass through the gate</t>
+          <t>Last required arrangement: Confirmed</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
         <is>
-          <t>After step 1 the status is Safety Review and the log shows both the earlier approval and the new submission; the event is not Confirmed until step 3 completes</t>
+          <t>The Event enters Safety Review automatically and the Safety Officer is notified; no Coordinator submission action is required; the Activity log still shows the earlier safety approval and the new move into Safety Review; the earlier decision is not reused, so the Event stays in Safety Review until a Safety Officer decides again</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(attendee): record Aaron's E09-S04 manual run with screenshots (SCRUM-224)
TC_E09S04_01 to _05 all PASS on the local real stack at bb64b9e, ten
screenshots (T-93). Exports the test-case workbook as CAA 311026 for
TC_E09S04_04's new wording.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES.xlsx
+++ b/docs/testing/PROJECT TEST CASES.xlsx
@@ -16407,7 +16407,8 @@
       <c r="H305" s="2" t="inlineStr">
         <is>
           <t>1. Log in as attendee_k@example.com
-  2. Open the registration page for the event of "Tech Conference 2026"</t>
+  2. Open the registration page for the event of "Tech Conference 2026"
+  3. Send a registration request</t>
         </is>
       </c>
       <c r="I305" s="2" t="inlineStr">
@@ -16417,7 +16418,7 @@
       </c>
       <c r="J305" s="2" t="inlineStr">
         <is>
-          <t>No waiting list option is offered; registration is simply shown as closed</t>
+          <t>No waiting list is offered; the Attendee can still request a place, which is saved as Pending for the Organiser to review (C-98, T-85)</t>
         </is>
       </c>
     </row>

</xml_diff>